<commit_message>
docs: remove editorial notes from submission files
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -11,24 +11,24 @@
     <sheet name="Nhật ký Thay đổi v1 sang v2" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Định nghĩa đo" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Gate 30-60-90" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Bằng chứng" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Kế hoạch dữ liệu" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dashboard Hành Động'!$A$4:$H$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Dashboard Hành Động'!$1:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Dashboard Hành Động'!$A$1:$H$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Nhật ký Thay đổi v1 sang v2'!$A$4:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Nhật ký Thay đổi v1 sang v2'!$A$4:$F$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Nhật ký Thay đổi v1 sang v2'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Nhật ký Thay đổi v1 sang v2'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Nhật ký Thay đổi v1 sang v2'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Định nghĩa đo'!$A$4:$E$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Định nghĩa đo'!$1:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Định nghĩa đo'!$A$1:$E$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Gate 30-60-90'!$A$4:$E$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Gate 30-60-90'!$1:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Gate 30-60-90'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Bằng chứng'!$A$4:$E$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Bằng chứng'!$1:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Bằng chứng'!$A$1:$E$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Kế hoạch dữ liệu'!$A$4:$E$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Kế hoạch dữ liệu'!$1:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Kế hoạch dữ liệu'!$A$1:$E$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -614,14 +614,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>DASHBOARD HÀNH ĐỘNG ÁP DỤNG AI — V2 HIỆU CHỈNH THEO YEUCAU.MD</t>
+          <t>DASHBOARD HÀNH ĐỘNG ÁP DỤNG AI — BẢN V2</t>
         </is>
       </c>
     </row>
     <row r="2" ht="56" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Promt Kiếm Tông | Baseline chưa có bằng chứng kèm theo; mọi mục tiêu là đề xuất, xác nhận tại Gate 30 | Xem Định nghĩa đo, Gate 30-60-90, Bằng chứng</t>
+          <t>Dự án: Trợ lý AI tra cứu quy trình &amp; chính sách nội bộ | Nhóm: Promt Kiếm Tông | Baseline thu thập tại Gate 30</t>
         </is>
       </c>
     </row>
@@ -653,7 +653,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Baseline / trạng thái</t>
+          <t>Mốc ban đầu (Baseline)</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="G4" s="13" t="inlineStr">
         <is>
-          <t>Owner nghiệp vụ cần xác nhận</t>
+          <t>Người phụ trách (Owner)</t>
         </is>
       </c>
       <c r="H4" s="13" t="inlineStr">
@@ -695,13 +695,13 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Đo tại Gate 30. Bản nhóm ghi 18%, chưa xác minh; kỳ đo và mẫu số chưa thống nhất. Không gọi đây là tỷ lệ adoption.</t>
+          <t>Thu thập tại Gate 30 từ log tác vụ và lịch phân công; ghi rõ số người sử dụng và số người có tác vụ đủ điều kiện.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Gate 30: khóa baseline.
-Gate 60/90: ≥85% người có tác vụ đủ điều kiện trong tuần. Đối chiếu số người thực tế, không suy từ 18% của 25 người.</t>
+Gate 60/90: ≥85% người có tác vụ đủ điều kiện trong tuần.</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
@@ -716,7 +716,7 @@
       </c>
       <c r="H5" s="14" t="inlineStr">
         <is>
-          <t>Dưới 85% ở Gate 60/90: trong 24 giờ làm việc kiểm lỗi truy cập, thiếu nguồn và điểm vướng với người chưa dùng; sửa/hỗ trợ trong workflow, đo lại tuần kế tiếp. Không nhắc tăng prompt.</t>
+          <t>Dưới 85% ở Gate 60/90: trong 24 giờ làm việc kiểm lỗi truy cập, thiếu nguồn và điểm vướng với người chưa dùng; sửa/hỗ trợ trong workflow, đo lại tuần kế tiếp.</t>
         </is>
       </c>
     </row>
@@ -738,7 +738,7 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Đo tại Gate 30. Bản nhóm ghi 22%, chưa có mẫu/log kiểm chứng.</t>
+          <t>Thu thập tại Gate 30 từ log hoàn tất, hỏi thêm và làm lại; theo dõi thêm 2 ngày làm việc.</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>Đo ≥50 lượt thủ công tương đương tại Gate 30. Bản nhóm ghi 8,5 phút, chưa xác minh.</t>
+          <t>Đo ≥50 lượt tra cứu thủ công tương đương tại Gate 30, phân theo loại tác vụ và độ khó.</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>QA đo tại Gate 30. Bản nhóm ghi 0%, chưa có tập đánh giá; thiếu dữ liệu không đồng nghĩa 0%.</t>
+          <t>QA đo tại Gate 30 trên bộ câu hỏi kiểm thử, đối chiếu nội dung, điều khoản và hiệu lực nguồn.</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>Đo tại Gate 30. Bản nhóm ghi 0%, chưa có log. Không có ca cần chuyển thì N/A, không ghi 100%.</t>
+          <t>Thu thập tại Gate 30 từ log định tuyến và kiểm thử các ca cần chuyển người. Không phát sinh ca thực tế: N/A.</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="H9" s="14" t="inlineStr">
         <is>
-          <t>Bỏ sót/thiếu ngữ cảnh/quá 4 giờ: chuyển thủ công ngay và báo Chủ quy trình; rà định tuyến, cảnh báo và hàng đợi trong 24 giờ làm việc. Thiếu/mâu thuẫn/hết hiệu lực nguồn, ngoài phạm vi hoặc nghi sai đều là trigger, không dùng điểm tự tin 85%.</t>
+          <t>Bỏ sót/thiếu ngữ cảnh/quá 4 giờ: chuyển thủ công ngay và báo Chủ quy trình; rà định tuyến, cảnh báo và hàng đợi trong 24 giờ làm việc. Thiếu/mâu thuẫn/hết hiệu lực nguồn, ngoài phạm vi hoặc nghi sai đều kích hoạt chuyển người.</t>
         </is>
       </c>
     </row>
@@ -910,13 +910,13 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Chưa xác định; khóa baseline và lưu lượng tại Gate 30. Không tự đặt 0 giờ khi chưa đo.</t>
+          <t>Xác định tại Gate 30 từ baseline thời gian, lưu lượng tác vụ và công sức QA/hỗ trợ/bảo trì.</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
           <t>Gate 30: xác nhận lưu lượng và tính khả thi.
-Gate 60/90: ≥120 giờ ròng/tháng trên một tháng đủ dữ liệu. Đây là mục tiêu, chưa phải kết quả/ROI.</t>
+Gate 60/90: ≥120 giờ ròng/tháng trên một tháng đủ dữ liệu.</t>
         </is>
       </c>
       <c r="F10" s="15" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>Dưới 120 giờ/tháng: so khối lượng, công sức và baseline, sửa rồi đo lại, chưa mở rộng. Nếu ròng ≤0 trong 4 tuần đủ mẫu sau một vòng sửa, trình đề xuất dừng. Không cắt QA để làm đẹp số.</t>
+          <t>Dưới 120 giờ/tháng: so khối lượng, công sức và baseline, sửa rồi đo lại, chưa mở rộng. Nếu ròng ≤0 trong 4 tuần đủ mẫu sau một vòng sửa, trình đề xuất dừng.</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CPromt Kiếm Tông | V2 hiệu chỉnh | Trang &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;CPromt Kiếm Tông | Dashboard v2 | Trang &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -961,7 +961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -975,14 +975,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>ĐỐI CHIẾU V1 → V2 — GIỮ NGUYÊN FILE V1</t>
+          <t>ĐỐI CHIẾU THAY ĐỔI GIỮA DASHBOARD V1 VÀ V2</t>
         </is>
       </c>
     </row>
     <row r="2" ht="56" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Góp ý Nhóm 05 theo bản nhóm ghi, chưa kèm biên bản. Các sửa rà soát bổ sung không được gán thành góp ý Nhóm 05.</t>
+          <t>Nhóm: Promt Kiếm Tông | Các thay đổi về chỉ số, bàn giao, nguồn đo và trách nhiệm sau phản biện chéo</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1049,12 @@
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Theo bản nhóm: prompt cao/Like không chứng minh chất lượng; cần biên bản xác nhận.</t>
+          <t>Số prompt cao và lượt Like không chứng minh chất lượng kết quả.</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>Chuyển sang chất lượng và kết quả thực của workflow; không gọi activity là vô dụng trong mọi mục đích.</t>
+          <t>Đo chất lượng và kết quả của workflow để hỗ trợ quyết định triển khai.</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>Theo bản nhóm: cần chốt chặn khi câu hỏi phức tạp hoặc nguồn thiếu; chưa kèm biên bản.</t>
+          <t>Cần điểm bàn giao khi câu hỏi phức tạp hoặc nguồn thiếu.</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
@@ -1113,12 +1113,12 @@
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Theo bản nhóm: chỉ số cần nguồn thực tế; cần xác nhận nội dung phản biện nhận về.</t>
+          <t>Chỉ số cần nguồn dữ liệu có thể đối chiếu trong workflow.</t>
         </is>
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>Chưa có baseline thì không báo kết quả. 120 giờ/tháng là mục tiêu đề xuất.</t>
+          <t>Đánh giá mục tiêu 120 giờ tiết kiệm ròng/tháng từ log tác vụ và công sức bổ sung.</t>
         </is>
       </c>
     </row>
@@ -1145,49 +1145,18 @@
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>Theo bản nhóm: hành động cần owner/thời hạn; cần biên bản.</t>
+          <t>Hành động cần owner và thời hạn xử lý cụ thể.</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Phân biệt vai trò đơn vị vận hành với thành viên điều phối bài nhóm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="170" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Hiệu chỉnh theo yêu cầu 16/10/2026</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>Các file v2 cũ lệch target, kỳ đo 18%, mô tả 65%; thiếu nguồn số liệu.</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>Thống nhất 6 chỉ số/5 tầng; ghi chưa xác minh, định nghĩa mẫu/gate; bỏ confidence 85% và accuracy 99% chưa kiểm định.</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>Rà soát bổ sung theo Yeucau.md; không gán cho Nhóm 05.</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>V1 không sửa. Cần nhóm bổ sung case thực tế và bằng chứng trước khi xác nhận đạt toàn bộ đề bài.</t>
-        </is>
-      </c>
-    </row>
+          <t>Xác định trách nhiệm dữ liệu, kiểm tra chất lượng và xử lý ngoại lệ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="170" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A4:F9"/>
+  <autoFilter ref="A4:F8"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -1197,7 +1166,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CPromt Kiếm Tông | V2 hiệu chỉnh | Trang &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;CPromt Kiếm Tông | Dashboard v2 | Trang &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1232,7 +1201,7 @@
     <row r="2" ht="56" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Mục tiêu đề xuất, baseline chờ xác nhận. Ngưỡng gate phải đồng thời đạt; thiếu dữ liệu không coi là đạt.</t>
+          <t>Công thức, mẫu đo và cách xử lý dữ liệu thiếu cho sáu chỉ số trong dashboard</t>
         </is>
       </c>
     </row>
@@ -1288,12 +1257,12 @@
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Mẫu số=0 → N/A. Quy mô 25 theo bài nhóm, phải xác nhận; không suy số người từ 18%.</t>
+          <t>Mẫu số bằng 0: N/A. Ghi số người thực tế và dùng cùng định nghĩa trong mọi kỳ đo.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Chủ quy trình xác nhận phạm vi và ngày đo tại Gate 30. Đây là usage trong workflow, không phải adoption.</t>
+          <t>Chủ quy trình khóa phạm vi và kỳ đo tại Gate 30; mức dùng được theo dõi theo tuần.</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1412,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CPromt Kiếm Tông | V2 hiệu chỉnh | Trang &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;CPromt Kiếm Tông | Dashboard v2 | Trang &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1478,7 +1447,7 @@
     <row r="2" ht="56" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Vai trò nghiệp vụ cần được đơn vị xác nhận; sinh viên chỉ điều phối bài nhóm. Mục tiêu phải xác nhận ở Gate 30.</t>
+          <t>Mỗi gate có owner, bằng chứng và điều kiện chuyển; mục tiêu được phê duyệt tại Gate 30.</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1498,12 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Xác nhận case thật; khóa phạm vi/nguồn, bổ nhiệm owner; duyệt quyền, ngân sách, hỗ trợ và nơi lưu log. Baseline ≥50 lượt thủ công tương đương; bộ thử ≥100 câu gồm ≥20 ca cần chuyển.</t>
+          <t>Khóa phạm vi/nguồn, bổ nhiệm owner; duyệt quyền, ngân sách, hỗ trợ và nơi lưu log. Baseline ≥50 lượt thủ công tương đương; bộ thử ≥100 câu gồm ≥20 ca cần chuyển.</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Trích nguồn ≥95%; bàn giao đúng 100% ca thử; đủ baseline/owner/nguồn lực; không lỗi nghiêm trọng chưa xử lý. Mức dùng, hành vi, thời gian và giờ ròng: khóa baseline/kiểm tính khả thi, chưa đặt kết quả đã đạt.</t>
+          <t>Trích nguồn ≥95%; bàn giao đúng 100% ca thử; đủ baseline/owner/nguồn lực; không lỗi nghiêm trọng chưa xử lý. Mức dùng, hành vi, thời gian và giờ ròng: khóa baseline và kiểm tra tính khả thi.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -1588,7 +1557,7 @@
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>Đạt đủ → đề xuất mở rộng từng đợt sau phê duyệt; không tự đặt quy mô 200 người hoặc tuyên bố normalization.</t>
+          <t>Đạt đủ điều kiện: trình phê duyệt mở rộng từng đợt theo ngân sách và năng lực vận hành.</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -1608,7 +1577,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CPromt Kiếm Tông | V2 hiệu chỉnh | Trang &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;CPromt Kiếm Tông | Dashboard v2 | Trang &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1623,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1636,14 +1605,14 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>TRẠNG THÁI BẰNG CHỨNG VÀ VIỆC CẦN NHÓM BỔ SUNG</t>
+          <t>KẾ HOẠCH THU THẬP DỮ LIỆU VÀ NGUỒN THAM KHẢO</t>
         </is>
       </c>
     </row>
     <row r="2" ht="56" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Nhóm xác nhận chưa có bằng chứng kèm theo khi rà soát. Không công bố log nhạy cảm; dùng bản tổng hợp đã ẩn danh.</t>
+          <t>Thu thập baseline trong giai đoạn 0–30 ngày; tổng hợp hằng tuần và đánh giá giá trị theo tháng.</t>
         </is>
       </c>
     </row>
@@ -1662,216 +1631,190 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>Hiện có</t>
+          <t>Dữ liệu cần thu thập</t>
         </is>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>Trạng thái</t>
+          <t>Thời điểm / cỡ mẫu</t>
         </is>
       </c>
       <c r="D4" s="16" t="inlineStr">
         <is>
-          <t>Cần bổ sung / giới hạn</t>
+          <t>Cách đối chiếu</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>Người điều phối</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="170" customHeight="1">
+          <t>Người phụ trách</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>Case thực tế và 25 người</t>
+          <t>Mức dùng</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Mô tả tình huống trong bài nhóm; chưa có căn cứ đính kèm.</t>
+          <t>Người có tác vụ AI gắn ticket; người được phân công tác vụ đủ điều kiện.</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Chưa xác minh</t>
+          <t>Gate 30 khóa baseline; tổng hợp hằng tuần.</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>Xác nhận tình huống từ lớp/doanh nghiệp; nguồn ghi nhận, thời điểm, phạm vi. Không dùng case tưởng tượng theo §3.1.</t>
+          <t>Đối chiếu log tác vụ với lịch phân công, ghi cả tử số và mẫu số.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
         <is>
-          <t>Trần Đình Hinh điều phối; Chủ quy trình xác nhận.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="170" customHeight="1">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>18% quay lại</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>README: sau 2 tuần; memo cũ: sau 4 tuần; Excel cũ: tuần 1.</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>Chưa xác minh; không khớp kỳ đo, thiếu tử/mẫu số</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>Định nghĩa quay lại, ngày đo và số người đủ điều kiện. 18% không tương ứng số nguyên người trên 25; không sửa thành số mới khi thiếu log.</t>
-        </is>
-      </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>Trần Đình Hinh điều phối, đối chiếu log.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="170" customHeight="1">
+          <t>Chủ quy trình Vận hành</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Hành vi và năng suất</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Trạng thái hoàn tất/duyệt; hỏi thêm, làm lại; phút lao động từng đoạn và loại tác vụ.</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Baseline ≥50 lượt thủ công; pilot ≥50 tác vụ đủ theo dõi/tuần, cộng 2 ngày theo dõi sửa.</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Đối chiếu ticket_id, loại/độ khó và thời gian từng đoạn; cộng công sức chuyển/làm lại.</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Chủ quy trình Vận hành</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="150" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>8,5 phút; 22%; trích nguồn/handoff 0%</t>
+          <t>Chất lượng trích nguồn</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Có số trong bản nhóm, chưa có tập đo.</t>
+          <t>Câu trả lời, link văn bản, điều khoản, hiệu lực và kết quả chấm QA.</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>Chưa xác minh; baseline hiện tại phải đo lại/xác nhận</t>
+          <t>Gate 30: ≥100 câu thử, gồm ≥20 ca cần chuyển; vận hành QA ngẫu nhiên ≥50 câu/tuần hoặc toàn bộ nếu ít hơn.</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>Log tác vụ đã ẩn danh, phương pháp đo theo Định nghĩa đo; thiếu dữ liệu không suy ra 0%.</t>
+          <t>QA đối chiếu nguồn chuẩn; ca rủi ro kiểm riêng ngoài mẫu ngẫu nhiên.</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>Đinh Xuân Quyền tổng hợp; Hoàng Quốc Dũng cùng QA đối chiếu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="170" customHeight="1">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>65%; 450 phiên; phỏng vấn 10/10</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>Các bản mô tả khác nhau về kỳ và tiêu chí bỏ dở; chưa có log/ghi nhận.</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>Chưa xác minh; không dùng làm kết quả đã chứng minh</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>Đính kèm bản tổng hợp có ngày, mẫu, định nghĩa, câu hỏi phỏng vấn và người tổng hợp; không tự tạo lời trích dẫn.</t>
-        </is>
-      </c>
-      <c r="E8" s="15" t="inlineStr">
-        <is>
-          <t>Nhóm trưởng xác nhận với người thu thập.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="170" customHeight="1">
+          <t>QA; AI Tech Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Bàn giao</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Lý do chuyển, ngữ cảnh, ticket_id, người nhận và thời điểm tạo/nhận.</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Toàn bộ ca cần chuyển và bộ thử Gate 30.</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Rà ca được gắn cờ cùng ca bỏ sót do QA phát hiện; so SLA 4 giờ làm việc.</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Chủ quy trình Vận hành; AI Tech Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="150" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>Phản biện Nhóm 05</t>
+          <t>Giá trị</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Có mô tả góp ý trong bài, chưa kèm biên bản.</t>
+          <t>Lưu lượng theo loại tác vụ, phút baseline/thực tế, công sức QA/bảo trì/hỗ trợ tăng thêm.</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>Theo bài nhóm ghi; chưa xác minh</t>
+          <t>Gate 30 kiểm tính khả thi; Gate 60/90 dùng một tháng đủ dữ liệu.</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>Ghi riêng góp ý đã đưa đi và ≥2 góp ý nhận về, người tham gia và sửa tương ứng. V1 được giữ nguyên để đối chiếu.</t>
+          <t>Tính giờ ròng theo Định nghĩa đo; không cộng trùng công sức đã tính trong tác vụ.</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Nhóm trưởng xác nhận.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="170" customHeight="1">
-      <c r="A10" s="15" t="inlineStr">
+          <t>Chủ quy trình Vận hành</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Case tham khảo Morgan Stanley</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>https://openai.com/index/morgan-stanley/</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Đã kiểm tra nguồn ngày 16/10/2026</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>Nguồn mô tả eval trước triển khai, chuyên gia chấm, QA hồi quy và người kiểm. Hỗ trợ lựa chọn thiết kế, không xác nhận hiện trạng nội bộ hoặc quan hệ nhân quả riêng của citations.</t>
-        </is>
-      </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>Suy luận áp dụng của nhóm, không phải log doanh nghiệp nhóm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="170" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Mục tiêu ≥120 giờ/tháng</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>Chưa có baseline, lưu lượng và công sức tăng thêm.</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>Mục tiêu đề xuất; chưa phải kết quả/ROI</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>Kiểm định lượng tác vụ và phút tiết kiệm ròng; chốt mục tiêu có thể thu thập và nguồn lực tại Gate 30.</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>Chủ quy trình Vận hành phê duyệt.</t>
-        </is>
-      </c>
-    </row>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Nguồn tham khảo về đánh giá và kiểm soát chất lượng AI.</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Bài học áp dụng: đánh giá trước triển khai, chuyên gia chấm, QA hồi quy và người kiểm đầu ra.</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Nhóm Promt Kiếm Tông</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="170" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A4:E11"/>
+  <autoFilter ref="A4:E10"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
@@ -1884,7 +1827,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;CPromt Kiếm Tông | V2 hiệu chỉnh | Trang &amp;P / &amp;N</oddFooter>
+    <oddFooter>&amp;CPromt Kiếm Tông | Dashboard v2 | Trang &amp;P / &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>